<commit_message>
Add About/Career pages and unify navigation
Introduces full `about.html` and `career.html` pages with new branded content, sections, and CTAs. Updates existing pages to route About and Career links to these dedicated pages, removes legacy investor-focused nav items, and aligns footer/mobile drawer links across the site. Adds shared frontend support for career application UX in `script.js` (career modal, role prefill, file upload/drag-drop validation, submission toast) and extensive new styling in `style.css` for the About and Career experiences. Also adds EmailJS CDN loading to key pages and updates the business workbook asset.
</commit_message>
<xml_diff>
--- a/SIDDBC.xlsx
+++ b/SIDDBC.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6981ca84042a0c22/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\plit04\Downloads\Sidhu Website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="222" documentId="8_{9474C0A5-497C-428B-852B-8FB27E64F43D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C47D86B1-E7DE-4E40-9A07-6F431514F9BE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B729840A-ABAA-4A59-84A8-84772CEAD3B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{207EEDE1-94DA-47B6-AEAB-B7B758AC4833}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{207EEDE1-94DA-47B6-AEAB-B7B758AC4833}"/>
   </bookViews>
   <sheets>
     <sheet name="Our services" sheetId="1" r:id="rId1"/>
@@ -242,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -260,19 +260,18 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -608,14 +607,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{361EE8B7-BC46-4D3C-AB38-40B3FC8E5441}">
   <dimension ref="A1:J57"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="59.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="2.88671875" style="11" customWidth="1"/>
-    <col min="3" max="8" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="59.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="2.85546875" customWidth="1"/>
+    <col min="3" max="8" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="23.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="24" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -623,265 +622,267 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
       <c r="J3" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-    </row>
-    <row r="5" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C5" s="9" t="s">
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+    </row>
+    <row r="5" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
       <c r="J5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-    </row>
-    <row r="7" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
+    <row r="6" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+    </row>
+    <row r="7" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
       <c r="J7" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="C8" s="7" t="s">
+    <row r="8" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C9" s="10" t="s">
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C9" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
       <c r="J9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C10" s="9" t="s">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C10" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-    </row>
-    <row r="11" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+    </row>
+    <row r="11" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
       <c r="J11" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="C12" s="7" t="s">
+    <row r="12" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="C12" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C13" s="10" t="s">
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C13" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
       <c r="J13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C14" s="9" t="s">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C14" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-    </row>
-    <row r="15" spans="1:10" ht="18" x14ac:dyDescent="0.3">
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+    </row>
+    <row r="15" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
       <c r="J15" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-    </row>
-    <row r="17" spans="10:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+    </row>
+    <row r="17" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J17" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="10:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="10:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="J21" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="10:10" ht="18" x14ac:dyDescent="0.3">
+    <row r="23" spans="10:10" ht="18" x14ac:dyDescent="0.25">
       <c r="J23" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="10:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J25" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="10:10" ht="18" x14ac:dyDescent="0.3">
+    <row r="27" spans="10:10" ht="18" x14ac:dyDescent="0.25">
       <c r="J27" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="10:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J29" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="10:10" ht="18" x14ac:dyDescent="0.3">
+    <row r="31" spans="10:10" ht="18" x14ac:dyDescent="0.25">
       <c r="J31" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="33" spans="10:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J33" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="10:10" ht="18" x14ac:dyDescent="0.3">
+    <row r="35" spans="10:10" ht="18" x14ac:dyDescent="0.25">
       <c r="J35" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="10:10" x14ac:dyDescent="0.3">
+    <row r="37" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J37" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="39" spans="10:10" ht="18" x14ac:dyDescent="0.3">
+    <row r="39" spans="10:10" ht="18" x14ac:dyDescent="0.25">
       <c r="J39" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="10:10" x14ac:dyDescent="0.3">
+    <row r="41" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J41" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="10:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="45" spans="10:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="J45" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="10:10" ht="18" x14ac:dyDescent="0.3">
+    <row r="47" spans="10:10" ht="18" x14ac:dyDescent="0.25">
       <c r="J47" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="49" spans="10:10" x14ac:dyDescent="0.3">
+    <row r="49" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J49" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="51" spans="10:10" ht="18" x14ac:dyDescent="0.3">
+    <row r="51" spans="10:10" ht="18" x14ac:dyDescent="0.25">
       <c r="J51" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="10:10" x14ac:dyDescent="0.3">
+    <row r="53" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J53" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="55" spans="10:10" ht="18" x14ac:dyDescent="0.3">
+    <row r="55" spans="10:10" ht="18" x14ac:dyDescent="0.25">
       <c r="J55" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="10:10" x14ac:dyDescent="0.3">
+    <row r="57" spans="10:10" x14ac:dyDescent="0.25">
       <c r="J57" t="s">
         <v>27</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="C14:H16"/>
+    <mergeCell ref="C9:H9"/>
     <mergeCell ref="C4:H4"/>
     <mergeCell ref="C13:H13"/>
     <mergeCell ref="C8:H8"/>
@@ -889,8 +890,6 @@
     <mergeCell ref="C12:H12"/>
     <mergeCell ref="C5:H7"/>
     <mergeCell ref="C10:H11"/>
-    <mergeCell ref="C14:H16"/>
-    <mergeCell ref="C9:H9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -899,139 +898,139 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD831632-446A-4952-8CFC-D58E015266B3}">
   <dimension ref="A1:A57"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="23.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="24" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" ht="18" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" ht="18" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="18" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" ht="18" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="18" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" ht="18" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:1" ht="18" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" ht="18" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:1" ht="18" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" ht="18" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:1" ht="18" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:1" ht="18" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="39" spans="1:1" ht="18" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:1" ht="18" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="1:1" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:1" ht="18" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:1" ht="18" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="51" spans="1:1" ht="18" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:1" ht="18" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="55" spans="1:1" ht="18" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:1" ht="18" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>27</v>
       </c>

</xml_diff>